<commit_message>
docs: update data file for certificate portal
</commit_message>
<xml_diff>
--- a/certificate-portal/data.xlsx
+++ b/certificate-portal/data.xlsx
@@ -1,26 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shrut\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1D6097-D1AF-4B0C-9882-DBB60E1CFDF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView windowWidth="29400" windowHeight="11920"/>
   </bookViews>
   <sheets>
     <sheet name="Form Responses 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="88">
   <si>
     <t>Timestamp</t>
   </si>
@@ -281,38 +288,384 @@
   </si>
   <si>
     <t>IET DAVV</t>
+  </si>
+  <si>
+    <t>it.richajain@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="m/d/yyyy\ h:mm:ss"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="5">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="m/d/yyyy\ h:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="22">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -320,42 +673,319 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="4">
-    <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF5B3F86"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF5B3F86"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF5B3F86"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF5B3F86"/>
-        </bottom>
-      </border>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -380,35 +1010,48 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF5B3F86"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF5B3F86"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF5B3F86"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF5B3F86"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1">
-    <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+    <tableStyle name="Form Responses 1-style" pivot="0" count="4" xr9:uid="{D0363560-389F-ACCC-6AC2-096AB214F51C}">
+      <tableStyleElement type="wholeTable" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Form_Responses" displayName="Form_Responses" ref="A1:F28">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Form_Responses" displayName="Form_Responses" ref="A1:F28">
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Timestamp"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Email Address"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Name"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Google Email ID"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Institute"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Table number"/>
+    <tableColumn id="1" name="Timestamp"/>
+    <tableColumn id="2" name="Email Address"/>
+    <tableColumn id="3" name="Name"/>
+    <tableColumn id="4" name="Google Email ID"/>
+    <tableColumn id="5" name="Institute"/>
+    <tableColumn id="6" name="Table number"/>
   </tableColumns>
   <tableStyleInfo name="Form Responses 1-style" showFirstColumn="1" showLastColumn="1" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -606,22 +1249,21 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr defaultColWidth="12.6339285714286" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="5"/>
   <cols>
-    <col min="1" max="12" width="18.90625" customWidth="1"/>
+    <col min="1" max="12" width="18.9107142857143" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22.5" customHeight="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -641,9 +1283,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" ht="22.5" customHeight="1" spans="1:6">
       <c r="A2" s="2">
-        <v>46143.43597604167</v>
+        <v>46143.4359760417</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>6</v>
@@ -661,9 +1303,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" ht="22.5" customHeight="1" spans="1:6">
       <c r="A3" s="2">
-        <v>46143.439009965281</v>
+        <v>46143.4390099653</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>9</v>
@@ -681,9 +1323,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" ht="22.5" customHeight="1" spans="1:6">
       <c r="A4" s="2">
-        <v>46143.439346898143</v>
+        <v>46143.4393468981</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>12</v>
@@ -701,9 +1343,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="22.5" customHeight="1" spans="1:6">
       <c r="A5" s="2">
-        <v>46143.436502870369</v>
+        <v>46143.4365028704</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>16</v>
@@ -721,9 +1363,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="22.5" customHeight="1" spans="1:6">
       <c r="A6" s="2">
-        <v>46143.438444444444</v>
+        <v>46143.4384444444</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>20</v>
@@ -741,9 +1383,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="22.5" customHeight="1" spans="1:6">
       <c r="A7" s="2">
-        <v>46143.439149166668</v>
+        <v>46143.4391491667</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>23</v>
@@ -761,9 +1403,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="22.5" customHeight="1" spans="1:6">
       <c r="A8" s="2">
-        <v>46143.439516898143</v>
+        <v>46143.4395168981</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>26</v>
@@ -781,9 +1423,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="22.5" customHeight="1" spans="1:6">
       <c r="A9" s="2">
-        <v>46143.420815717589</v>
+        <v>46143.4208157176</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>29</v>
@@ -801,9 +1443,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="22.5" customHeight="1" spans="1:6">
       <c r="A10" s="2">
-        <v>46143.422103368051</v>
+        <v>46143.4221033681</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>32</v>
@@ -821,9 +1463,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" ht="22.5" customHeight="1" spans="1:6">
       <c r="A11" s="2">
-        <v>46143.422634039351</v>
+        <v>46143.4226340394</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>35</v>
@@ -841,9 +1483,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" ht="22.5" customHeight="1" spans="1:6">
       <c r="A12" s="2">
-        <v>46143.420740277783</v>
+        <v>46143.4207402778</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>38</v>
@@ -861,9 +1503,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" ht="22.5" customHeight="1" spans="1:6">
       <c r="A13" s="2">
-        <v>46143.463050104168</v>
+        <v>46143.4630501042</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>41</v>
@@ -881,9 +1523,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" ht="22.5" customHeight="1" spans="1:6">
       <c r="A14" s="2">
-        <v>46143.466023460649</v>
+        <v>46143.4660234606</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>45</v>
@@ -901,9 +1543,9 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" ht="22.5" customHeight="1" spans="1:6">
       <c r="A15" s="2">
-        <v>46143.435039247684</v>
+        <v>46143.4350392477</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>48</v>
@@ -921,9 +1563,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" ht="22.5" customHeight="1" spans="1:6">
       <c r="A16" s="2">
-        <v>46143.441118159724</v>
+        <v>46143.4411181597</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>51</v>
@@ -941,9 +1583,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" ht="22.5" customHeight="1" spans="1:6">
       <c r="A17" s="2">
-        <v>46143.442788460648</v>
+        <v>46143.4427884606</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>53</v>
@@ -961,9 +1603,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" ht="22.5" customHeight="1" spans="1:6">
       <c r="A18" s="2">
-        <v>46143.435389583334</v>
+        <v>46143.4353895833</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>56</v>
@@ -981,9 +1623,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" ht="22.5" customHeight="1" spans="1:6">
       <c r="A19" s="2">
-        <v>46143.436841770832</v>
+        <v>46143.4368417708</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>59</v>
@@ -1001,9 +1643,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" ht="22.5" customHeight="1" spans="1:6">
       <c r="A20" s="2">
-        <v>46143.454572349539</v>
+        <v>46143.4545723495</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>61</v>
@@ -1021,9 +1663,9 @@
         <v>8</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" ht="22.5" customHeight="1" spans="1:6">
       <c r="A21" s="2">
-        <v>46143.470421782404</v>
+        <v>46143.4704217824</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>63</v>
@@ -1041,9 +1683,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" ht="22.5" customHeight="1" spans="1:6">
       <c r="A22" s="2">
-        <v>46143.63395802083</v>
+        <v>46143.6339580208</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>66</v>
@@ -1061,9 +1703,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" ht="22.5" customHeight="1" spans="1:6">
       <c r="A23" s="2">
-        <v>46143.635145787033</v>
+        <v>46143.635145787</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>70</v>
@@ -1081,9 +1723,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" ht="22.5" customHeight="1" spans="1:6">
       <c r="A24" s="2">
-        <v>46143.635760023149</v>
+        <v>46143.6357600231</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>73</v>
@@ -1101,9 +1743,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" ht="22.5" customHeight="1" spans="1:6">
       <c r="A25" s="2">
-        <v>46143.670816990736</v>
+        <v>46143.6708169907</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>75</v>
@@ -1121,9 +1763,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" ht="22.5" customHeight="1" spans="1:6">
       <c r="A26" s="2">
-        <v>46143.670986631943</v>
+        <v>46143.6709866319</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>78</v>
@@ -1141,9 +1783,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" ht="22.5" customHeight="1" spans="1:6">
       <c r="A27" s="2">
-        <v>46143.67182452546</v>
+        <v>46143.6718245255</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>80</v>
@@ -1161,9 +1803,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" ht="22.5" customHeight="1" spans="1:6">
       <c r="A28" s="2">
-        <v>46143.672391817134</v>
+        <v>46143.6723918171</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>84</v>
@@ -1181,8 +1823,33 @@
         <v>1</v>
       </c>
     </row>
+    <row r="29" customFormat="1" ht="22.5" customHeight="1" spans="1:6">
+      <c r="A29" s="2">
+        <v>46143.4359760417</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F29" s="3">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B29" r:id="rId2" display="it.richajain@gmail.com"/>
+    <hyperlink ref="D29" r:id="rId2" display="it.richajain@gmail.com"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>